<commit_message>
new data has been added to the excel file
</commit_message>
<xml_diff>
--- a/data/airflow.xlsx
+++ b/data/airflow.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\githubdemo\apache-airflow\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42B249FF-3038-402D-9BD6-38CFE19A3A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F18D202-89E1-43CB-8CC8-8B421E3ED246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4934DE36-DB61-4546-B575-AA784025563D}"/>
   </bookViews>
@@ -39,20 +39,58 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t xml:space="preserve">number </t>
-  </si>
-  <si>
-    <t xml:space="preserve">name </t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+  <si>
+    <t>order_id</t>
+  </si>
+  <si>
+    <t>product</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>Uzbekistan</t>
+  </si>
+  <si>
+    <t>Mouse</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>Kazakhstan</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Headphones</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -80,8 +118,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,30 +466,109 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9C1DDDB-15BE-43B7-B176-FB9B665FA6EC}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2">
+    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1">
+        <v>800</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
+      <c r="B3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1">
+        <v>25</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3</v>
+      </c>
+      <c r="D4" s="1">
+        <v>50</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1">
+        <v>300</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1">
+        <v>80</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
the etl has been done
</commit_message>
<xml_diff>
--- a/data/airflow.xlsx
+++ b/data/airflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\githubdemo\apache-airflow\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F18D202-89E1-43CB-8CC8-8B421E3ED246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC10202-4929-4016-B920-C805A3CD5859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4934DE36-DB61-4546-B575-AA784025563D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
   <si>
     <t>order_id</t>
   </si>
@@ -466,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9C1DDDB-15BE-43B7-B176-FB9B665FA6EC}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -571,6 +571,23 @@
         <v>9</v>
       </c>
     </row>
+    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1">
+        <v>25</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
new spark files are added and the compose docker file is edited to run the pyspark
</commit_message>
<xml_diff>
--- a/data/airflow.xlsx
+++ b/data/airflow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\githubdemo\apache-airflow\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC10202-4929-4016-B920-C805A3CD5859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2A33C6-4CF8-4086-BBD8-8E9A80C4F0B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4934DE36-DB61-4546-B575-AA784025563D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
   <si>
     <t>order_id</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t>Headphones</t>
+  </si>
+  <si>
+    <t>j</t>
   </si>
 </sst>
 </file>
@@ -466,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9C1DDDB-15BE-43B7-B176-FB9B665FA6EC}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -588,6 +591,23 @@
         <v>6</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1">
+        <v>12</v>
+      </c>
+      <c r="D8" s="1">
+        <v>45</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>